<commit_message>
Rebuild Mode 5 Golden Path doc with fresh Playwright run on mbx-ee-dev
Fresh dedicated fixture (E2E Mode5 Fresh Test material) exercises the
Produce FG wizard on top of the new native-MO Slab-cutting mechanism
(13 Sep 2026 rebuild) for the first time end to end, covering both the
G2b (must produce) and G2a (surplus stock, no production needed)
branches, invoicing, payment, and journal items.
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode5.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode5.xlsx
@@ -9,10 +9,9 @@
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="G1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="G2a" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="G2b" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="G3" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="G4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="G2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="G3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="G4" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C2:D13"/>
+  <dimension ref="C2:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="2" max="2"/>
@@ -485,14 +484,14 @@
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 12</t>
+          <t>Total test cases: 13</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 9 / 3 / 0</t>
+          <t>High / Medium / Low: 10 / 3 / 0</t>
         </is>
       </c>
     </row>
@@ -511,7 +510,7 @@
     <row r="9">
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>G1 — ขาย (Sale — Mode 5, FG Production)</t>
+          <t>G1 — ขาย (Sale — สินค้าสำเร็จรูปที่ต้องผลิตจาก Slab)</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -521,41 +520,31 @@
     <row r="10">
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>G2a — ผลิต — กรณี FG มีสต็อกพอแล้ว (ไม่ต้องผลิตซ้ำ)</t>
+          <t>G2 — ผลิต — กรณี FG ไม่มี/ไม่พอในสต็อก (ต้องผลิตจริง)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>G2b — ผลิต — กรณี FG ไม่มี/ไม่พอในสต็อก (ต้องผลิตจริง)</t>
+          <t>G3 — จัดส่ง + ขายซ้ำ — กรณี FG มีสต็อกพอแล้ว (ไม่ต้องผลิตซ้ำ)</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>G3 — จัดส่ง (Delivery)</t>
+          <t>G4 — บัญชี (Accounting + Payment)</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>G4 — บัญชี (Accounting)</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -589,7 +578,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>G1. ขาย (Sale — Mode 5, FG Production) — ADR-029 — เพิ่มบรรทัดสินค้าสำเร็จรูป (FG) แล้วยืนยันคำสั่งขาย</t>
+          <t>G1. ขาย (Sale — สินค้าสำเร็จรูปที่ต้องผลิตจาก Slab) — ADR-029 — ขายสินค้า FG (เช่น Countertop) ที่ยังไม่ได้ผลิตจริงได้เลย</t>
         </is>
       </c>
     </row>
@@ -663,37 +652,35 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เพิ่มบรรทัดสินค้าสำเร็จรูป (FG) ในใบสั่งขาย</t>
+          <t>เพิ่มบรรทัดสินค้า FG (Finished Good) ใน Sale Order ใหม่</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มี Slab (วัตถุดิบตั้งต้นของ FG นี้) อยู่ในสต็อกที่ไหนสักแห่งแล้ว (ไม่จำเป็นต้องว่าง — ระบบจะเช็คให้เองตอน Confirm)</t>
+          <t>มี Slab พร้อมอยู่แล้วในสต็อกที่สถานีผลิต (Stone Production) จาก Material ที่ตั้งค่า FG ไว้ (มี Block/Slab/FG ครบ 3 สินค้า)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Sales &gt; Orders &gt; New
 2. เลือกลูกค้า
-3. เพิ่มบรรทัด เลือกสินค้าสำเร็จรูป (FG)
-4. กรอกจำนวนที่ต้องการขาย</t>
+3. เพิ่มบรรทัด เลือกสินค้า FG ของ Material นั้น</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
           <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
-สินค้า = "Carrara White - Countertop"
-จำนวน = 3</t>
+สินค้า = E2E Mode5 Fresh Test - Countertop</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เพิ่มบรรทัดสำเร็จ ราคาต่อหน่วยขึ้นตามราคาตั้งต้นของสินค้า — ตัวอย่างจริง: 15,000.00 บาท/หน่วย × 3 = 45,000.00 + VAT 7% = 48,150.00 บาท</t>
+          <t>เพิ่มบรรทัดสำเร็จ ราคาต่อหน่วยขึ้นเป็นราคาตั้งต้นของสินค้า FG (ตัวอย่างจริง: 8,500/หน่วย)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H4" s="7" t="n"/>
@@ -710,7 +697,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>ยืนยัน (Confirm) Sale Order</t>
+          <t>ยืนยัน (Confirm) Sale Order — ยังไม่มี FG ในสต็อกเลย</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -730,7 +717,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order เกิด Delivery Order อัตโนมัติ 1 ใบ — ถ้า FG ที่ขายมีสต็อกว่างพอ บรรทัดจะไม่มีปุ่ม "Produce FG" เลย (ไปต่อที่ G2a) แต่ถ้าไม่พอ ปุ่ม "Cut to Order"/"Produce FG" จะปรากฏให้กดต่อ (ไปต่อที่ G2b) — ตัวอย่างจริง (กรณีสต็อกไม่พอ): S00112 ยอดรวม 48,150.00 บาท, ปุ่ม Produce FG ปรากฏที่บรรทัด</t>
+          <t>SO เปลี่ยนสถานะเป็น Sales Order ยอดรวม 9,095.00 บาท (รวม VAT) — บรรทัดสินค้า FG ปรากฏลิงก์ "Produce FG" ให้กดเพื่อผลิต เพราะยังไม่มีสต็อก FG เลย — ตัวอย่างจริง: S00127</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -758,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -778,7 +765,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>G2a. ผลิต — กรณี FG มีสต็อกพอแล้ว (ไม่ต้องผลิตซ้ำ) — ระบบเช็คสต็อกว่างของ FG เองก่อนเสมอ — เพิ่งแก้ไขให้ถูกต้อง 2026-09-07</t>
+          <t>G2. ผลิต — กรณี FG ไม่มี/ไม่พอในสต็อก (ต้องผลิตจริง) — ADR-029, stone.fg.production.wizard — เปิด wizard "Produce FG" ตัดจาก Slab ที่มีอยู่</t>
         </is>
       </c>
     </row>
@@ -852,28 +839,27 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>ระบบข้ามขั้นตอนผลิต เมื่อ FG มีสต็อกว่างพออยู่แล้ว</t>
+          <t>เปิด wizard "Produce FG" — ระบบจับคู่ Slab ที่จะใช้ให้อัตโนมัติ</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>สินค้า FG ตัวนี้มีสต็อกว่าง (ไม่ถูกจองไปกับออเดอร์อื่น) พอกับจำนวนที่จะขาย</t>
+          <t>ทำ TC-E2E-M5-02 เสร็จแล้ว มี Slab พร้อมอยู่ที่สถานีผลิตแล้ว (ย้ายด้วย Internal Transfer ล่วงหน้า)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เพิ่มบรรทัดสินค้า FG ในใบสั่งขายเหมือน TC-E2E-M5-01
-2. กด Confirm เหมือน TC-E2E-M5-02</t>
+          <t>1. กดลิงก์ "Produce FG" บนบรรทัดสินค้า FG ของ Sale Order</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>สินค้า = "Carrara White - Countertop" จำนวน = 2 (ตอนนั้นมีสต็อกว่างเหลือ 4 หน่วยจากการผลิตเผื่อไว้ใน G2b)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดไม่มีปุ่ม "Produce FG" ปรากฏเลย (ต่างจาก TC-E2E-M5-02) และไม่ขึ้นแถวในหน้า Factory Worklist เลย — ไปต่อที่การจัดส่งได้ทันทีโดยไม่ต้องผลิตอะไรเพิ่ม — ตัวอย่างจริง: S00113 ยอดรวม 32,100.00 บาท</t>
+          <t>เปิด wizard สำเร็จ ช่อง "Slab to Consume" เติมให้อัตโนมัติเป็น Slab ตัวแรกที่มี Material ตรงกันและสถานะ Available (v1: จับคู่ตาม Material อย่างเดียว) พร้อมบรรทัดผลผลิตเริ่มต้น 1 บรรทัดตรงกับสินค้าที่ขาย จำนวน 1 — ตัวอย่างจริง: Slab BLK-26-0029 #1</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -881,15 +867,100 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>✅ เพิ่งแก้ไข 2026-09-07: ก่อนหน้านี้ระบบไม่เคยเช็คสต็อกของ FG เอง จะขึ้นเตือนให้ผลิตซ้ำทุกครั้งแม้มี FG เหลือพอขายอยู่แล้ว — ตอนนี้เช็คให้อัตโนมัติแล้วจากสต็อก "ว่างจริง" ที่ไม่ถูกจองไปกับออเดอร์อื่น</t>
-        </is>
-      </c>
+      <c r="H4" s="7" t="n"/>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
       <c r="L4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-04</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>ปรับจำนวนผลผลิตแล้วกด "Produce" — สร้าง Manufacturing Order</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-03 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>1. แก้ไขจำนวนในบรรทัดผลผลิตจาก 1 เป็น 2
+2. กดปุ่ม "Produce"</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>จำนวนผลผลิต = 2</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>สร้าง Manufacturing Order สำเร็จ ยืนยันอัตโนมัติทันที (Confirmed) ระบบเติม Bill of Material ให้อัตโนมัติจาก FG Material ที่เลือก จำนวนที่จะผลิต = 2.00 Slab ที่เลือกถูกจับจองเป็นวัตถุดิบ (To Consume 1.00, Available) ผูกกับบรรทัด SO เดิม ("For Sale Order Line") — ตัวอย่างจริง: EG01/STFG/00015</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>ผลผลิตต่อ Slab กำหนดตอนผลิตจริง ไม่ใช่อัตราตายตัว (ADR-029) — เคสนี้ตั้งใจผลิต 2 หน่วยจาก Slab เดียว แม้บรรทัด SO ต้องการแค่ 1 หน่วย เพื่อเผื่อสต็อกไว้ขายลูกค้ารายถัดไป (ดู TC-E2E-M5-07)</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-05</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>กด "Complete FG Production" — ได้สินค้า FG จริงเข้าสต็อก</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-04 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "Complete FG Production" บน Manufacturing Order</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Manufacturing Order เสร็จสมบูรณ์ (สถานะ Done) จำนวนที่ผลิตจริง = 2.00/2.00 ได้ Lot/Serial ใหม่ของสินค้า FG (ตัวอย่างจริง: FG-EG01/STFG/00015) Slab ที่ใช้เป็นวัตถุดิบเปลี่ยนสถานะเป็น Consumed หมดสภาพขายต่อ สินค้า FG 2 หน่วยเข้าสต็อกจริง</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -900,6 +971,243 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>G3. จัดส่ง + ขายซ้ำ — กรณี FG มีสต็อกพอแล้ว (ไม่ต้องผลิตซ้ำ) — ส่งของบรรทัดแรก แล้วขายลูกค้าใหม่ด้วยสต็อกส่วนเกินที่เหลือ ไม่ต้องผ่าน wizard อีก</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-06</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>จัดส่งใบส่งของของบรรทัดแรก (SO1)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-05 เสร็จแล้ว มีสินค้า FG พร้อมส่งแล้ว</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติของ S00127
+2. กดปุ่ม Validate</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จทันที (จองสต็อกไว้ให้แล้วตั้งแต่ผลิตเสร็จ) — ตัวอย่างจริง: EG01/OUT/00081</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-07</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>สร้าง Sale Order ใหม่ขายสินค้า FG ตัวเดียวกันอีกครั้ง — ใช้สต็อกส่วนเกิน</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-06 เสร็จแล้ว มีสินค้า FG เหลือในสต็อก 1 หน่วยจากการผลิตครั้งก่อน</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิด Sales &gt; Orders &gt; New
+2. เลือกลูกค้าเดิม
+3. เพิ่มบรรทัด เลือกสินค้า FG ตัวเดียวกัน จำนวน 1
+4. กด Confirm</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
+สินค้า = E2E Mode5 Fresh Test - Countertop
+จำนวน = 1</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>SO ยืนยันสำเร็จ ยอดรวม 9,095.00 บาทเท่าเดิม ใบส่งของที่เกิดขึ้นอัตโนมัติจองสต็อก (Reserved/Assigned) ได้ทันทีจากสต็อกส่วนเกินที่เหลือ โดยไม่ต้องเปิด "Produce FG" เลย — ตัวอย่างจริง: S00128</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>✨ พฤติกรรมจริงที่พบ: ลิงก์ "Produce FG" ยังปรากฏอยู่บนบรรทัดเสมอ ไม่ว่าสต็อกจะพอหรือไม่ — จุดต่างจริงของ G2a คือ "ไม่จำเป็นต้องกด" เพราะใบส่งของจองสต็อกสำเร็จได้เองทันที ไม่ใช่ว่าลิงก์หายไป</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-08</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>จัดส่งใบส่งของของบรรทัดที่สอง (SO2)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-07 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติของ S00128
+2. กดปุ่ม Validate</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จทันที เหมือนกับ TC-E2E-M5-06 ทุกประการ — ตัวอย่างจริง: EG01/OUT/00082</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -925,7 +1233,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>G2b. ผลิต — กรณี FG ไม่มี/ไม่พอในสต็อก (ต้องผลิตจริง) — ย้าย Slab เข้าสถานีผลิต แล้วเปิด wizard "Produce FG" ตัด/ผลิตจริง</t>
+          <t>G4. บัญชี (Accounting + Payment) — ออกใบแจ้งหนี้ทั้ง 2 ใบ + รับชำระเงิน + ตรวจรายการบัญชี (COGS ต้องไม่เป็น 0)</t>
         </is>
       </c>
     </row>
@@ -994,22 +1302,24 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-04</t>
+          <t>TC-E2E-M5-09</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เห็นคิวงานที่หน้า Factory Worklist</t>
+          <t>ออกใบแจ้งหนี้บรรทัดแรก (SO1)</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-02 เสร็จแล้ว (กรณีสต็อกไม่พอ)</t>
+          <t>ทำ TC-E2E-M5-06 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดเมนู Stone Slab &gt; Tools &gt; Factory Worklist</t>
+          <t>1. เปิด Sale Order S00127 &gt; กดปุ่ม "Create Invoice"
+2. เลือก "Regular Invoice" &gt; Create Draft Invoice
+3. กด Confirm บนใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1019,12 +1329,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เห็นแถวของ SO นี้ขึ้นคิวงาน คอลัมน์ "ต้องทำ" ระบุ "รอผลิต FG (Cut to Order / Produce FG)" — ตัวอย่างจริง: S00112, สินค้า Carrara White - Countertop, จำนวน 3.00</t>
+          <t>ใบแจ้งหนี้ยืนยันสำเร็จ สถานะ Posted ยอดรวม 9,095.00 บาท (รวม VAT) — ตัวอย่างจริง: INV/2026/00031</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H4" s="7" t="n"/>
@@ -1036,36 +1346,34 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-05</t>
+          <t>TC-E2E-M5-10</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>ย้าย Slab (วัตถุดิบของ FG) เข้าสถานีผลิต</t>
+          <t>ออกใบแจ้งหนี้บรรทัดที่สอง (SO2)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>มี Slab ของ Material เดียวกับ FG นี้ อยู่ที่ Location "Stone Available"</t>
+          <t>ทำ TC-E2E-M5-08 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Inventory &gt; Internal Transfers &gt; New
-2. ตั้งต้นทาง (Source Location) = Stone Available
-3. ตั้งปลายทาง (Destination Location) = Stone Production
-4. เพิ่มสินค้า Slab ของ Material นั้น จำนวน 1
-5. กด Validate</t>
+          <t>1. เปิด Sale Order S00128 &gt; กดปุ่ม "Create Invoice"
+2. เลือก "Regular Invoice" &gt; Create Draft Invoice
+3. กด Confirm บนใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>สินค้า = "Carrara White - Slab" จำนวน = 1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบโอนย้ายเปลี่ยนสถานะเป็น Done Slab ถูกย้ายเข้า Stone Production เรียบร้อย พร้อมให้ผลิตต่อ — ตัวอย่างจริง: EG01/INT/00053 (Slab BDL-00002 #8)</t>
+          <t>ใบแจ้งหนี้ยืนยันสำเร็จ สถานะ Posted ยอดรวม 9,095.00 บาทเท่ากับใบแรกทุกประการ (ราคาขายเท่ากัน) — ตัวอย่างจริง: INV/2026/00032</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1082,23 +1390,22 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-06</t>
+          <t>TC-E2E-M5-11</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>เปิด wizard "Produce FG" — ระบบจับคู่ Slab ให้อัตโนมัติ</t>
+          <t>ตรวจรายการบัญชีของใบแจ้งหนี้ (Journal Items) — ต้นทุนขาย (COGS) ต้องไม่เป็น 0</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-05 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-09 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กลับไปที่บรรทัดสินค้า FG ใน Sale Order
-2. กดปุ่ม "Produce FG"</t>
+          <t>1. เปิด Customer Invoice &gt; กดแท็บ "Journal Items"</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1108,7 +1415,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>หน้าต่าง Produce FG เปิดขึ้น ช่อง "Slab to Consume" ถูกเติมชื่อ Slab ที่เพิ่งย้ายเข้าสถานีผลิตให้อัตโนมัติ (ไม่ต้องเลือกเอง) พร้อมบรรทัดผลผลิต 1 บรรทัดตรงกับสินค้าที่ขายอยู่แล้ว — ตัวอย่างจริง: Slab to Consume = BDL-00002 #8</t>
+          <t>เห็นรายการครบ 5 บรรทัด สมดุลกันทั้ง 2 ฝั่ง (เดบิต = เครดิต) พร้อม Analytic Distribution ผูกกับ Material/Block ทุกบรรทัด — ตัวอย่างจริง INV/2026/00031: เครดิต "411150 Sales Revenue - FG Production" 8,500.00, เครดิต "213200 Output VAT" 595.00, เดบิต "112100 Trade Receivables" 9,095.00, เครดิต "113150 Inventory - Stone FG (Finished Goods)" 375.00, เดบิต "511100 Cost of Goods Sold" 375.00 — รวมสมดุล 9,470.00 = 9,470.00 (COGS ไม่ใช่ 0 บาท ตัดจริงตามบัญชีที่ถูกต้อง)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1125,45 +1432,41 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-07</t>
+          <t>TC-E2E-M5-12</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>กรอกจำนวนผลผลิตจริงจาก Slab นี้ แล้วกดผลิต</t>
+          <t>บันทึกรับชำระเงินใบแจ้งหนี้บรรทัดแรก (SO1)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-06 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-09 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. แก้จำนวนในบรรทัดผลผลิตเป็นจำนวนที่ตัด/ผลิตได้จริงจาก Slab นี้
-2. กดปุ่ม "Produce"</t>
+          <t>1. เปิดใบแจ้งหนี้ &gt; กดปุ่ม "Pay"
+2. เลือกวิธีชำระเงินที่ต้องการ &gt; กดยืนยัน</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>จำนวนผลผลิต = 6 (ลูกค้าสั่งแค่ 3 — ตัดเผื่อสต็อกไว้ขายรอบหน้าด้วย)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>เกิดใบสั่งผลิต (Manufacturing Order) ใหม่ ผูก Slab ที่เลือกเป็นวัตถุดิบ จำนวนที่ต้องผลิตตรงกับที่กรอก — ตัวอย่างจริง: EG01/STFG/00012 (To Produce 6.00)</t>
+          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" ทันที — ตัวอย่างจริง: INV/2026/00031</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>1 Slab ตัดออกมาได้กี่ชิ้นไม่ตายตัว — ฝ่ายผลิตกรอกจำนวนจริงที่ตัดได้ตอนนี้เอง ไม่ต้องเท่ากับจำนวนที่ลูกค้าสั่งพอดี (ตัดเผื่อสต็อกไว้ขายออเดอร์ถัดไปได้)</t>
-        </is>
-      </c>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
@@ -1172,23 +1475,23 @@
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-08</t>
+          <t>TC-E2E-M5-13</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>กด "Complete FG Production" — ปิดงานผลิต</t>
+          <t>บันทึกรับชำระเงินใบแจ้งหนี้บรรทัดที่สอง (SO2)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-07 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-10 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบสั่งผลิตที่เพิ่งสร้าง
-2. กดปุ่ม "Complete FG Production"</t>
+          <t>1. เปิดใบแจ้งหนี้ &gt; กดปุ่ม "Pay"
+2. เลือกวิธีชำระเงินที่ต้องการ &gt; กดยืนยัน</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1198,12 +1501,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>ใบสั่งผลิตเปลี่ยนสถานะเป็น Done Slab ที่ใช้ถูกตัดออกจากสต็อกจนหมด (ใช้ครั้งเดียว ไม่เหลือให้ใช้ซ้ำ) FG เข้าสต็อกจริงตามจำนวนที่ผลิต พร้อม Lot ใหม่ — ตัวอย่างจริง: EG01/STFG/00012 ผลิตสำเร็จ 6.00/6.00 ได้ Lot "FG-EG01/STFG/00012"</t>
+          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" ทันทีเหมือนกัน — ตัวอย่างจริง: INV/2026/00032</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1211,384 +1514,6 @@
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>G3. จัดส่ง (Delivery) — ทั้ง 2 กรณี (ผลิตใหม่ / มีสต็อกอยู่แล้ว) ส่งมอบแบบเดียวกัน ไม่มีการดักสแกน Serial</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>TC ID</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Precondition</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Status (Pass/Fail)</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-09</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>ส่งมอบสินค้าที่เพิ่งผลิตเสร็จ (กรณี G2b)</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-08 เสร็จแล้ว มีใบส่งของอัตโนมัติรออยู่ตั้งแต่ตอน Confirm</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิด Inventory &gt; Deliveries
-2. เปิดใบส่งของของ SO นี้
-3. กด Validate</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done — ไม่มีการดักสแกน Serial เหมือนสินค้า Block/Slab (ส่งได้ทันทีเมื่อสต็อกพร้อม) — ตัวอย่างจริง: EG01/OUT/00066 (Carrara White - Countertop 3.00/3.00 พร้อมส่ง)</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-10</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>ส่งมอบสินค้าที่ไม่ต้องผลิต (กรณี G2a)</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-03 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิด Inventory &gt; Deliveries
-2. เปิดใบส่งของของ SO นี้
-3. กด Validate</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done ทันที ดึงสต็อกจาก FG ที่มีอยู่แล้วโดยไม่ผ่านขั้นตอนผลิตเลยสักครั้ง — ตัวอย่างจริง: EG01/OUT/00067 (Carrara White - Countertop 2.00/2.00)</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>G4. บัญชี (Accounting) — ออกใบแจ้งหนี้ &amp; ตรวจรายการบัญชี</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>TC ID</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Precondition</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Status (Pass/Fail)</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-11</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>ออกใบแจ้งหนี้และยืนยัน (Post)</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-09 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิด Sale Order &gt; กด "Create Invoice"
-2. เลือก "Regular invoice" &gt; กด "Create Draft Invoice"
-3. เปิดใบแจ้งหนี้ที่เกิดขึ้น &gt; กด Confirm</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดตรงกับ SO เป๊ะ — ตัวอย่างจริง: INV/2026/00018 (48,150.00 บาท จาก S00112)</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-12</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>ตรวจรายการบัญชีของใบแจ้งหนี้ (Journal Items) — ยืนยันว่าลง COGS ถูกต้อง</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-11 เสร็จแล้ว (ตัวอย่างนี้ใช้ SO/Invoice อีกใบที่ขายจาก FG ล็อตใหม่ล้วน เพื่อให้เห็นรายการ COGS จริง)</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิดใบแจ้งหนี้ &gt; กดแท็บ "Journal Items"</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) พร้อมมีรายการ COGS ปรากฏครบ — ตัวอย่างจริง: INV/2026/00020 (SO S00114, ขาย FG ล็อตใหม่ 2 หน่วย) เดบิต Trade Receivables 32,100.00 = เครดิต Sales Revenue - FG Production 30,000.00 + Output VAT 2,100.00 บาท และมีคู่ COGS แยกสมดุลกันเอง: เดบิต 511100 Cost of Goods Sold 933.33 = เครดิต 113150 Inventory - Stone FG 933.33 บาท (933.33 = 466.67 บาท/หน่วย × 2 หน่วย ตรงกับต้นทุน Slab จริงเป๊ะ)</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>ℹ️ หมายเหตุ: ใบแจ้งหนี้ของ S00112/S00113 เองไม่มีรายการ COGS ขึ้นมา — ตอนแรกเข้าใจผิดว่าเป็นบั๊ก แต่ตรวจสอบลึกแล้วพบว่าไม่ใช่: หินที่ส่งมอบ 5 หน่วยในนั้นตรงกับสต็อกเก่าที่มีอยู่แล้ว 5 หน่วยพอดี ซึ่งเป็นข้อมูลสาธิตเก่าที่มีมูลค่าบันทึกไว้ 0.00 บาทตั้งแต่ต้น (ช่องว่างข้อมูลที่รู้และยอมรับไว้แล้วก่อนหน้านี้ ไม่ใช่ปัญหาใหม่) ระบบคิดต้นทุนแบบ FIFO จึงตัดจากของเก่า (มูลค่า 0) ก่อนของใหม่ที่เพิ่งผลิตถูกต้องแล้วตามหลัก FIFO — ไม่ใช่บั๊กของ Mode 5 เลย ดูตัวอย่างที่ยืนยันว่าระบบลงบัญชีถูกต้องจริงด้านล่าง (ใช้ของใหม่ล้วน ไม่ปนของเก่า)</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Rebuild Golden Path Mode 5 (v3): Standard + new Custom variant (ADR-068)
Standard (ADR-067): "Produce FG" now creates a draft MO directly, no
wizard popup — FG Output tab replaces the old wizard's qty field.

Custom (ADR-068, first Golden Path coverage — no v1/v2 predecessor):
Stage 2 "Cutting Plan" (Slab -> N pieces sharing 1 lot) then Stage 3
"Assembly" via the extended stone.custom.bom.wizard (pick a Cutting
Plan Lot instead of/alongside BOQ components).

13 test cases, both flows run live end-to-end on mbx-ee-dev with real
document numbers and balanced accounting (Standard 10,110.00, Custom
12,916.89). Cross-linked from library.html/archived.html — Mode 4
remains the only pending-rebuild entry.
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode5.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode5.xlsx
@@ -11,7 +11,6 @@
     <sheet name="G1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="G2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="G3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="G4" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C2:D12"/>
+  <dimension ref="C2:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="2" max="2"/>
@@ -470,7 +469,7 @@
     <row r="2">
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>EMG-O — Test Cases: E2E Flow — Mode 5 (Stone Production / FG Production)</t>
+          <t>EMG-O — Test Cases: E2E Flow — Mode 5 (Slab → Finished Goods)</t>
         </is>
       </c>
     </row>
@@ -491,7 +490,7 @@
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 10 / 3 / 0</t>
+          <t>High / Medium / Low: 11 / 2 / 0</t>
         </is>
       </c>
     </row>
@@ -510,41 +509,31 @@
     <row r="9">
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>G1 — ขาย (Sale — สินค้าสำเร็จรูปที่ต้องผลิตจาก Slab)</t>
+          <t>G1 — เตรียมแผ่น (Slab) ก่อนผลิต — เหมือน Mode 3 ทุกประการ</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>G2 — ผลิต — กรณี FG ไม่มี/ไม่พอในสต็อก (ต้องผลิตจริง)</t>
+          <t>G2 — ขาย + ผลิต — สินค้า FG มาตรฐาน (Standard, เช่น Countertop)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>G3 — จัดส่ง + ขายซ้ำ — กรณี FG มีสต็อกพอแล้ว (ไม่ต้องผลิตซ้ำ)</t>
+          <t>G3 — ขาย + ผลิต — งาน Custom สั่งทำพิเศษ (ADR-068, เช่น เจดีย์บัว/ซุ้มบัว)</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>G4 — บัญชี (Accounting + Payment)</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -558,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -578,7 +567,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>G1. ขาย (Sale — สินค้าสำเร็จรูปที่ต้องผลิตจาก Slab) — ADR-029 — ขายสินค้า FG (เช่น Countertop) ที่ยังไม่ได้ผลิตจริงได้เลย</t>
+          <t>G1. เตรียมแผ่น (Slab) ก่อนผลิต — เหมือน Mode 3 ทุกประการ — ตัด Block เป็น Slab ล่วงหน้า ก่อนขายจริง — reuse กลไกเดียวกับ Mode 3 (Block-to-Slab) ไม่มีอะไรใหม่</t>
         </is>
       </c>
     </row>
@@ -652,30 +641,31 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เพิ่มบรรทัดสินค้า FG (Finished Good) ใน Sale Order ใหม่</t>
+          <t>ตัด Block เป็น Slab ไว้ล่วงหน้า (ยังไม่ผูกกับ SO ใดๆ)</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มี Slab พร้อมอยู่แล้วในสต็อกที่สถานีผลิต (Stone Production) จาก Material ที่ตั้งค่า FG ไว้ (มี Block/Slab/FG ครบ 3 สินค้า)</t>
+          <t>มี Block พร้อมอยู่แล้วในสต็อก (ยังไม่ตัด) จาก Material ที่ตั้งค่า Finished Good ไว้ครบ (มี Block/Slab/FG 3 สินค้า)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Sales &gt; Orders &gt; New
-2. เลือกลูกค้า
-3. เพิ่มบรรทัด เลือกสินค้า FG ของ Material นั้น</t>
+          <t>1. เปิด Manufacturing &gt; New
+2. เลือก Block ที่ต้องการตัด + กรอกขนาดที่ต้องการ
+3. ย้ายด่วน (Move to Production) &gt; Confirm &gt; ทำ Work Orders &gt; Complete Cut</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
-สินค้า = E2E Mode5 Fresh Test - Countertop</t>
+          <t>Stone Block = BLK-26-0036
+Target Slab L (M) = 1.50
+Target Slab H (M) = 1.00</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เพิ่มบรรทัดสำเร็จ ราคาต่อหน่วยขึ้นเป็นราคาตั้งต้นของสินค้า FG (ตัวอย่างจริง: 8,500/หน่วย)</t>
+          <t>ได้แผ่นหินจริง 1 แผ่นเข้าสต็อก (ตัวอย่างจริง: BLK-26-0036 #1, 1.50 ตร.ม.) Block เหลือ CBM ส่วนที่ยังไม่ตัดไว้ขายต่อได้ (ตัวอย่างจริง: เหลือ 2.97 CBM จาก 3.00)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -683,53 +673,15 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>ใช้กลไกเดียวกับ Mode 3 (Block-to-Slab) เป๊ะๆ — Mode 5 ไม่มีขั้นตอนตัดของตัวเอง ต้องมี Slab พร้อมอยู่ในสต็อกก่อนเสมอ</t>
+        </is>
+      </c>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
       <c r="L4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-02</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>ยืนยัน (Confirm) Sale Order — ยังไม่มี FG ในสต็อกเลย</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-01 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>1. กดปุ่ม Confirm บน Sale Order</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order ยอดรวม 9,095.00 บาท (รวม VAT) — บรรทัดสินค้า FG ปรากฏลิงก์ "Produce FG" ให้กดเพื่อผลิต เพราะยังไม่มีสต็อก FG เลย — ตัวอย่างจริง: S00127</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -745,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -765,7 +717,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>G2. ผลิต — กรณี FG ไม่มี/ไม่พอในสต็อก (ต้องผลิตจริง) — ADR-029, stone.fg.production.wizard — เปิด wizard "Produce FG" ตัดจาก Slab ที่มีอยู่</t>
+          <t>G2. ขาย + ผลิต — สินค้า FG มาตรฐาน (Standard, เช่น Countertop) — ADR-029/067 — Produce FG สร้าง MO ตรงเลย ไม่ผ่าน wizard แล้ว</t>
         </is>
       </c>
     </row>
@@ -834,32 +786,36 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-03</t>
+          <t>TC-E2E-M5-02</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เปิด wizard "Produce FG" — ระบบจับคู่ Slab ที่จะใช้ให้อัตโนมัติ</t>
+          <t>เพิ่มบรรทัดสินค้า FG มาตรฐานใน Sale Order แล้ว Confirm</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-02 เสร็จแล้ว มี Slab พร้อมอยู่ที่สถานีผลิตแล้ว (ย้ายด้วย Internal Transfer ล่วงหน้า)</t>
+          <t>มี Slab พร้อมอยู่แล้วในสต็อกจาก TC-E2E-M5-01</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. กดลิงก์ "Produce FG" บนบรรทัดสินค้า FG ของ Sale Order</t>
+          <t>1. เปิด Sales &gt; Orders &gt; New
+2. เลือกลูกค้า
+3. เพิ่มบรรทัด เลือกสินค้า FG มาตรฐาน
+4. กด Confirm</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
+สินค้า = E2E Mode5 Fresh Test V2 - Countertop</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เปิด wizard สำเร็จ ช่อง "Slab to Consume" เติมให้อัตโนมัติเป็น Slab ตัวแรกที่มี Material ตรงกันและสถานะ Available (v1: จับคู่ตาม Material อย่างเดียว) พร้อมบรรทัดผลผลิตเริ่มต้น 1 บรรทัดตรงกับสินค้าที่ขาย จำนวน 1 — ตัวอย่างจริง: Slab BLK-26-0029 #1</t>
+          <t>SO ยืนยันสำเร็จ ยอดรวม 9,630.00 บาท (รวม VAT) บรรทัดสินค้า FG ปรากฏลิงก์ "Produce FG" เพราะยังไม่มีสต็อก FG เลย — ตัวอย่างจริง: S00137</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -876,33 +832,32 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-04</t>
+          <t>TC-E2E-M5-03</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>ปรับจำนวนผลผลิตแล้วกด "Produce" — สร้าง Manufacturing Order</t>
+          <t>กดลิงก์ "Produce FG" — ระบบสร้าง Manufacturing Order ตรงทันที ไม่มี wizard popup แล้ว</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-03 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-02 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. แก้ไขจำนวนในบรรทัดผลผลิตจาก 1 เป็น 2
-2. กดปุ่ม "Produce"</t>
+          <t>1. กดลิงก์ "Produce FG" บนบรรทัดสินค้า FG ของ Sale Order</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>จำนวนผลผลิต = 2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>สร้าง Manufacturing Order สำเร็จ ยืนยันอัตโนมัติทันที (Confirmed) ระบบเติม Bill of Material ให้อัตโนมัติจาก FG Material ที่เลือก จำนวนที่จะผลิต = 2.00 Slab ที่เลือกถูกจับจองเป็นวัตถุดิบ (To Consume 1.00, Available) ผูกกับบรรทัด SO เดิม ("For Sale Order Line") — ตัวอย่างจริง: EG01/STFG/00015</t>
+          <t>เปิดหน้า Manufacturing Order ฉบับร่างทันที (ไม่ใช่ popup) ช่อง Slab ที่ใช้ผลิตเติมให้อัตโนมัติเป็นแผ่นที่มี Material ตรงกันและสถานะ Available — ตัวอย่างจริง: MO EG01/STFG/00022, Slab BLK-26-0036 #1, ผูกกับ "For Sale Order Line" = S00137 ให้อัตโนมัติ</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -912,7 +867,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>ผลผลิตต่อ Slab กำหนดตอนผลิตจริง ไม่ใช่อัตราตายตัว (ADR-029) — เคสนี้ตั้งใจผลิต 2 หน่วยจาก Slab เดียว แม้บรรทัด SO ต้องการแค่ 1 หน่วย เพื่อเผื่อสต็อกไว้ขายลูกค้ารายถัดไป (ดู TC-E2E-M5-07)</t>
+          <t>✨ กลไกใหม่ (ADR-067, 14 ก.ย. 2026): เดิมกดแล้วเด้ง wizard ให้เลือก Slab/จำนวน ตอนนี้กดแล้วได้ MO ฉบับร่างเปิดขึ้นมาเลย ระบบจับคู่ Slab ที่ Material ตรงกันให้อัตโนมัติ ไม่ต้องเลือกเองก็ได้</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -923,22 +878,23 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-05</t>
+          <t>TC-E2E-M5-04</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>กด "Complete FG Production" — ได้สินค้า FG จริงเข้าสต็อก</t>
+          <t>ย้ายด่วน (Move to Production) แล้ว Confirm Manufacturing Order</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-04 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-03 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม "Complete FG Production" บน Manufacturing Order</t>
+          <t>1. กดปุ่ม "ย้ายด่วน (Move to Production)" บน MO
+2. กดปุ่ม Confirm</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -948,7 +904,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Manufacturing Order เสร็จสมบูรณ์ (สถานะ Done) จำนวนที่ผลิตจริง = 2.00/2.00 ได้ Lot/Serial ใหม่ของสินค้า FG (ตัวอย่างจริง: FG-EG01/STFG/00015) Slab ที่ใช้เป็นวัตถุดิบเปลี่ยนสถานะเป็น Consumed หมดสภาพขายต่อ สินค้า FG 2 หน่วยเข้าสต็อกจริง</t>
+          <t>Slab ถูกย้ายไปสถานีผลิต (Stone Production) สำเร็จ แล้ว Confirm ผ่านทันที ไม่มี error — สถานะ MO เปลี่ยนเป็น Confirmed</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -961,6 +917,139 @@
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-05</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>ทำ Work Order ให้เสร็จ แล้วบันทึกขนาดจริงในแท็บ "FG Output"</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-04 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>1. ไปแท็บ "Work Orders" กดเริ่ม/เสร็จตามลำดับจนครบ
+2. ไปแท็บ "FG Output" เพิ่มแถวขนาดจริงที่ตัดได้</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Width = 1.48, Length = 0.98, Thickness = 0.02, Qty = 1</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Work Orders ขึ้น Finished ครบ MO เปลี่ยนสถานะเป็น "To Close" แท็บ FG Output มี 1 แถวตามที่กรอก</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>✨ กลไกใหม่ (ADR-067): แท็บนี้แทนที่ wizard เดิมทั้งหมด — Factory กรอกขนาด/จำนวนที่ตัดได้จริงหลังตัดเสร็จ ตรงกับใบรายงานตัดกระดาษของโรงงานเป๊ะ ไม่มีคอลัมน์สินค้าเพราะทุกแถวนับรวมเป็นสินค้า FG ตัวเดียวของ MO นี้อยู่แล้ว</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-06</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>กด "Complete FG Production" — ได้สินค้า FG จริงเข้าสต็อก</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-05 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "Complete FG Production" บน Manufacturing Order</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>MO เสร็จสมบูรณ์ (สถานะ Done) ได้ Lot/Serial ใหม่ของสินค้า FG (ตัวอย่างจริง: FG-EG01/STFG/00022) Slab ที่ใช้เป็นวัตถุดิบเปลี่ยนสถานะเป็น Consumed สินค้า FG 1 หน่วยเข้าสต็อกจริง</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-07</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>จัดส่ง ออกใบแจ้งหนี้ และรับชำระเงิน (Standard)</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-06 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดใบส่งของที่เกิดขึ้นอัตโนมัติ &gt; Validate
+2. เปิด SO &gt; Create Invoice &gt; Regular Invoice &gt; Confirm
+3. เปิดใบแจ้งหนี้ &gt; Pay &gt; ยืนยันการชำระ</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของ Done (ตัวอย่างจริง: EG01/OUT/00091) ใบแจ้งหนี้ Posted ยอด 9,630.00 (ตัวอย่างจริง: INV/2026/00037) แล้วขึ้น In Payment — Journal Items 5 บรรทัด สมดุล 10,110.00 = 10,110.00 (COGS 480.00 ไม่ใช่ 0)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -976,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -996,7 +1085,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>G3. จัดส่ง + ขายซ้ำ — กรณี FG มีสต็อกพอแล้ว (ไม่ต้องผลิตซ้ำ) — ส่งของบรรทัดแรก แล้วขายลูกค้าใหม่ด้วยสต็อกส่วนเกินที่เหลือ ไม่ต้องผ่าน wizard อีก</t>
+          <t>G3. ขาย + ผลิต — งาน Custom สั่งทำพิเศษ (ADR-068, เช่น เจดีย์บัว/ซุ้มบัว) — ใหม่ทั้งหมด session นี้ — Stage 2 (ถอดแบบ) + Stage 3 (ประกอบ) สำหรับงานที่ไม่มี BOM ตายตัว</t>
         </is>
       </c>
     </row>
@@ -1065,33 +1154,38 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-06</t>
+          <t>TC-E2E-M5-08</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>จัดส่งใบส่งของของบรรทัดแรก (SO1)</t>
+          <t>Stage 2 — สร้าง "Cutting Plan" MO ถอดแบบ Slab เป็นชิ้นย่อย</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-05 เสร็จแล้ว มีสินค้า FG พร้อมส่งแล้ว</t>
+          <t>มี Slab พร้อมอยู่แล้วในสต็อก (แยกจาก Slab ที่ใช้ใน G2)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติของ S00127
-2. กดปุ่ม Validate</t>
+          <t>1. เปิด Manufacturing &gt; New
+2. เลือก "Source Slab (Cutting Plan)" เป็น Slab ที่จะถอดแบบ
+3. ไปแท็บ "Planned/Actual Pieces" เพิ่มแถวขนาดชิ้นที่ต้องการ
+4. ย้ายด่วน &gt; Confirm &gt; Work Orders &gt; "Complete Cutting Plan"</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Source Slab = BLK-26-0036 #2
+ชิ้นที่ 1: 0.25 x 0.20 m
+ชิ้นที่ 2: 0.20 x 0.15 m
+ชิ้นที่ 3: 0.15 x 0.10 m</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จทันที (จองสต็อกไว้ให้แล้วตั้งแต่ผลิตเสร็จ) — ตัวอย่างจริง: EG01/OUT/00081</t>
+          <t>MO เสร็จสมบูรณ์ (ตัวอย่างจริง: EG01/STCPL/00009) ได้ชิ้นงานจริง 3 ชิ้้น สถานะ "Staged (Cutting Plan WIP)" ทุกชิ้น — แชร์ Lot เดียวกันทั้งหมด (ตัวอย่างจริง: CUT-EG01/STCPL/00009, รวม 3.00 หน่วย) ชิ้นเหล่านี้จะไม่โผล่ในหน้า "Select Slabs" ของโหมดขายอื่นเลย เพราะยังไม่ใช่สต็อกขายได้จริง</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1099,7 +1193,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>✨ กลไกใหม่ทั้งหมด (ADR-068, session นี้): ใช้เมื่องานสั่งทำไม่มีสินค้า FG มาตรฐานให้เลือก ต้องเอา Slab มา "ถอดแบบ" เป็นชิ้นเล็กๆ ก่อน ทุกชิ้นจาก MO เดียวกันจะแชร์ Lot เดียวกัน (กันของปนกันตอนขนย้าย ไม่ใช่ QC รายชิ้น)</t>
+        </is>
+      </c>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
@@ -1108,272 +1206,36 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-07</t>
+          <t>TC-E2E-M5-09</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>สร้าง Sale Order ใหม่ขายสินค้า FG ตัวเดียวกันอีกครั้ง — ใช้สต็อกส่วนเกิน</t>
+          <t>สร้าง Sale Order ขายสินค้า Custom (ไม่มี FG มาตรฐานให้เลือก)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-06 เสร็จแล้ว มีสินค้า FG เหลือในสต็อก 1 หน่วยจากการผลิตครั้งก่อน</t>
+          <t>ทำ TC-E2E-M5-08 เสร็จแล้ว มี BOQ Document ผูกกับ Sale Order นี้ไว้ (จำเป็นสำหรับ wizard สร้าง BOM ในขั้นถัดไป)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Sales &gt; Orders &gt; New
-2. เลือกลูกค้าเดิม
-3. เพิ่มบรรทัด เลือกสินค้า FG ตัวเดียวกัน จำนวน 1
+          <t>1. เปิด Sales &gt; Orders &gt; New (ผูก BOQ Document)
+2. เลือกลูกค้า
+3. เพิ่มบรรทัด เลือกสินค้า Custom
 4. กด Confirm</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
           <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
-สินค้า = E2E Mode5 Fresh Test - Countertop
-จำนวน = 1</t>
+สินค้า = เจดีย์บัว S (Custom)</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>SO ยืนยันสำเร็จ ยอดรวม 9,095.00 บาทเท่าเดิม ใบส่งของที่เกิดขึ้นอัตโนมัติจองสต็อก (Reserved/Assigned) ได้ทันทีจากสต็อกส่วนเกินที่เหลือ โดยไม่ต้องเปิด "Produce FG" เลย — ตัวอย่างจริง: S00128</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>✨ พฤติกรรมจริงที่พบ: ลิงก์ "Produce FG" ยังปรากฏอยู่บนบรรทัดเสมอ ไม่ว่าสต็อกจะพอหรือไม่ — จุดต่างจริงของ G2a คือ "ไม่จำเป็นต้องกด" เพราะใบส่งของจองสต็อกสำเร็จได้เองทันที ไม่ใช่ว่าลิงก์หายไป</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-08</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>จัดส่งใบส่งของของบรรทัดที่สอง (SO2)</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-07 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติของ S00128
-2. กดปุ่ม Validate</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done สำเร็จทันที เหมือนกับ TC-E2E-M5-06 ทุกประการ — ตัวอย่างจริง: EG01/OUT/00082</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>G4. บัญชี (Accounting + Payment) — ออกใบแจ้งหนี้ทั้ง 2 ใบ + รับชำระเงิน + ตรวจรายการบัญชี (COGS ต้องไม่เป็น 0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>TC ID</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Precondition</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Status (Pass/Fail)</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-09</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>ออกใบแจ้งหนี้บรรทัดแรก (SO1)</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-06 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิด Sale Order S00127 &gt; กดปุ่ม "Create Invoice"
-2. เลือก "Regular Invoice" &gt; Create Draft Invoice
-3. กด Confirm บนใบแจ้งหนี้</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>ใบแจ้งหนี้ยืนยันสำเร็จ สถานะ Posted ยอดรวม 9,095.00 บาท (รวม VAT) — ตัวอย่างจริง: INV/2026/00031</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>TC-E2E-M5-10</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>ออกใบแจ้งหนี้บรรทัดที่สอง (SO2)</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>ทำ TC-E2E-M5-08 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>1. เปิด Sale Order S00128 &gt; กดปุ่ม "Create Invoice"
-2. เลือก "Regular Invoice" &gt; Create Draft Invoice
-3. กด Confirm บนใบแจ้งหนี้</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>ใบแจ้งหนี้ยืนยันสำเร็จ สถานะ Posted ยอดรวม 9,095.00 บาทเท่ากับใบแรกทุกประการ (ราคาขายเท่ากัน) — ตัวอย่างจริง: INV/2026/00032</t>
+          <t>SO ยืนยันสำเร็จ ยอดรวม 12,840.00 บาท (รวม VAT) บรรทัดสินค้าปรากฏลิงก์ "Produce FG" เหมือนเดิม แต่จะพาไปหน้าต่าง "สร้าง BOM จาก BOQ" แทน (ไม่ใช่สร้าง MO ตรงแบบ G2) เพราะสินค้านี้ไม่มี FG Raw Material ตายตัว — ตัวอย่างจริง: S00138</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1390,12 +1252,12 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-11</t>
+          <t>TC-E2E-M5-10</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ตรวจรายการบัญชีของใบแจ้งหนี้ (Journal Items) — ต้นทุนขาย (COGS) ต้องไม่เป็น 0</t>
+          <t>Stage 3 — กด "Produce FG" เปิด wizard "สร้าง BOM จาก BOQ" เลือก Cutting Plan Lot</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -1405,17 +1267,19 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Customer Invoice &gt; กดแท็บ "Journal Items"</t>
+          <t>1. กดลิงก์ "Produce FG" บนบรรทัดสินค้า
+2. เลือกช่อง "Cutting Plan Lot (Stage 2)" เป็น Lot จาก Stage 2
+3. กด "สร้าง BOM + MO"</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Cutting Plan Lot (Stage 2) = CUT-EG01/STCPL/00009</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็นรายการครบ 5 บรรทัด สมดุลกันทั้ง 2 ฝั่ง (เดบิต = เครดิต) พร้อม Analytic Distribution ผูกกับ Material/Block ทุกบรรทัด — ตัวอย่างจริง INV/2026/00031: เครดิต "411150 Sales Revenue - FG Production" 8,500.00, เครดิต "213200 Output VAT" 595.00, เดบิต "112100 Trade Receivables" 9,095.00, เครดิต "113150 Inventory - Stone FG (Finished Goods)" 375.00, เดบิต "511100 Cost of Goods Sold" 375.00 — รวมสมดุล 9,470.00 = 9,470.00 (COGS ไม่ใช่ 0 บาท ตัดจริงตามบัญชีที่ถูกต้อง)</t>
+          <t>สร้าง BOM + Manufacturing Order สำเร็จ แต่ MO ยังอยู่สถานะ Draft ให้ตรวจสอบก่อน (ต่างจากงาน Custom ที่ไม่ใช้ Cutting Plan Lot ซึ่งจะ Confirm ให้อัตโนมัติทันที) — ตัวอย่างจริง: EG01/STFG/00023 มีปุ่ม "Cutting Plan MO" เชื่อมกลับไปหา MO ของ Stage 2 ให้แล้ว</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1423,7 +1287,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>✨ ส่วนขยายใหม่ของ wizard เดิม (ADR-064 เดิม + ADR-068 เพิ่มเข้ามา): นอกจากเลือกวัสดุจาก BOQ ได้เหมือนเดิม ตอนนี้เลือก "Cutting Plan Lot (Stage 2)" ได้ด้วย — ระบบดึงมาทั้งก้อน (จำนวนเต็มของ Lot นั้น) ไม่ต้องกรอกจำนวนเอง</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
@@ -1432,23 +1300,23 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-12</t>
+          <t>TC-E2E-M5-11</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>บันทึกรับชำระเงินใบแจ้งหนี้บรรทัดแรก (SO1)</t>
+          <t>Confirm MO Stage 3 — ระบบเติมวัตถุดิบจาก Lot ให้อัตโนมัติ</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-09 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-10 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบแจ้งหนี้ &gt; กดปุ่ม "Pay"
-2. เลือกวิธีชำระเงินที่ต้องการ &gt; กดยืนยัน</t>
+          <t>1. ตรวจแท็บ "Components" ก่อน Confirm
+2. กดปุ่ม Confirm</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1458,12 +1326,12 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" ทันที — ตัวอย่างจริง: INV/2026/00031</t>
+          <t>แท็บ Components เติมแถววัตถุดิบจาก Cutting Plan Lot ให้อัตโนมัติ จำนวนเท่ากับที่มีอยู่เต็มก้อน (ตัวอย่างจริง: E2E Mode5 Fresh Test V2 - Cutting Plan WIP, 3.00 หน่วย) Confirm ผ่านสำเร็จ ไม่ต้องกรอกอะไรเพิ่มเอง</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -1475,23 +1343,22 @@
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>TC-E2E-M5-13</t>
+          <t>TC-E2E-M5-12</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>บันทึกรับชำระเงินใบแจ้งหนี้บรรทัดที่สอง (SO2)</t>
+          <t>ทำ MO ให้เสร็จด้วยปุ่ม Produce มาตรฐานของ Odoo (ไม่มีปุ่มเฉพาะ)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M5-10 เสร็จแล้ว</t>
+          <t>ทำ TC-E2E-M5-11 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบแจ้งหนี้ &gt; กดปุ่ม "Pay"
-2. เลือกวิธีชำระเงินที่ต้องการ &gt; กดยืนยัน</t>
+          <t>1. กรอกจำนวนที่ผลิตจริง &gt; กด Generate Lot ถ้ายังไม่มี &gt; กดปุ่ม Produce All</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1501,19 +1368,67 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ขึ้นสถานะ "In Payment" ทันทีเหมือนกัน — ตัวอย่างจริง: INV/2026/00032</t>
+          <t>MO เสร็จสมบูรณ์ (สถานะ Done) ได้สินค้า Custom 1 หน่วยเข้าสต็อกจริง ชิ้นงานทั้ง 3 ชิ้นจาก Stage 2 เปลี่ยนสถานะจาก "Staged" เป็น "Consumed" อัตโนมัติ (ไม่ค้างโชว์เป็น WIP อีกต่อไป) — กลับไปดูที่ MO ของ Stage 2 จะเห็นปุ่ม "Assembly MOs" เชื่อมมาที่ MO นี้แล้ว</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="n"/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>งาน Custom ใช้ปุ่ม Produce ธรรมดาของ Odoo เลย (ตาม ADR-064 เดิม "มาตรฐาน ODOO") ต่างจาก Stage 2/G2 ที่มีปุ่มเฉพาะของโมดูล</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M5-13</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>จัดส่ง ออกใบแจ้งหนี้ และรับชำระเงิน (Custom)</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M5-12 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดใบส่งของที่เกิดขึ้นอัตโนมัติ &gt; Validate
+2. เปิด SO &gt; Create Invoice &gt; Regular Invoice &gt; Confirm
+3. เปิดใบแจ้งหนี้ &gt; Pay &gt; ยืนยันการชำระ</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของ Done (ตัวอย่างจริง: EG01/OUT/00092) ใบแจ้งหนี้ Posted ยอด 12,840.00 (ตัวอย่างจริง: INV/2026/00038) แล้วขึ้น In Payment — Journal Items 5 บรรทัด สมดุล 12,916.89 = 12,916.89 (COGS 76.89 ไม่ใช่ 0)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>